<commit_message>
data: update 10 sources
</commit_message>
<xml_diff>
--- a/xlsx/BuxWV.xlsx
+++ b/xlsx/BuxWV.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="714">
   <si>
     <t>SORT</t>
   </si>
@@ -2001,9 +2001,6 @@
     <t>Violin, Viola da Gamba, Basso Continuo</t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
     <t>https://open.spotify.com/track/5V2jyo36dQEe0p4Cz9E8ci?si=847f7f58ae0045d0</t>
   </si>
   <si>
@@ -2021,6 +2018,9 @@
 6. Arioso</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/2aQJ1oNCXSL9XWiTuUnUh5?si=fd373831f91c4d53</t>
+  </si>
+  <si>
     <t>BuxWV 254</t>
   </si>
   <si>
@@ -2035,6 +2035,9 @@
 6. Presto</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/0FbNGIBKxiHuNKHwBVa3KV?si=be7fa4ab5bb44070</t>
+  </si>
+  <si>
     <t>BuxWV 255</t>
   </si>
   <si>
@@ -2044,6 +2047,9 @@
     <t>1. Vivace
 2. Lento
 3. Allegro</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/track/41snipsr88aJQUoHA5QzG3?si=85e3ec6881d14bfe</t>
   </si>
   <si>
     <t>BuxWV 256</t>
@@ -2057,6 +2063,9 @@
 3. Allegro
 4. Adagio
 5. Allegro</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/track/66Oq6njsbUCZu399cheY4q?si=3c2a19e57f834507</t>
   </si>
   <si>
     <t>BuxWV 257</t>
@@ -2071,6 +2080,9 @@
 4. Vivace
 5. Adagio
 6. Poco Presto</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/track/2A4yXz2VhLVEBHAv4EdEBv?si=351ec16a12b242af</t>
   </si>
   <si>
     <t>BuxWV 258</t>
@@ -2088,6 +2100,9 @@
 7. Prestissimo</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/0duf649xp9xw84aBwPsHKY?si=072c6e1d5f534488</t>
+  </si>
+  <si>
     <t>BuxWV 259</t>
   </si>
   <si>
@@ -2106,6 +2121,9 @@
 7. Presto</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/2MeB6etCEHNZixEffMDHV1?si=225bb02889a14429</t>
+  </si>
+  <si>
     <t>BuxWV 260</t>
   </si>
   <si>
@@ -2120,6 +2138,9 @@
 6. Vivace</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/1huvSof1V0V73f5FpE5RSI?si=9e8cb98ea5bc443c</t>
+  </si>
+  <si>
     <t>BuxWV 261</t>
   </si>
   <si>
@@ -2133,6 +2154,9 @@
 5. Gigue</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/3I9g7jkYe5sdW7DpIPdm55?si=d470f7acbb2640f2</t>
+  </si>
+  <si>
     <t>BuxWV 262</t>
   </si>
   <si>
@@ -2146,6 +2170,9 @@
 5. Vivace</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/3cBHUIZF9bPmf4DxkjOheq?si=f72f8f4b9f09441b</t>
+  </si>
+  <si>
     <t>BuxWV 263</t>
   </si>
   <si>
@@ -2157,6 +2184,9 @@
 3. Adagio
 4. Allegro
 5. Presto</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/track/2C5lNDTCyHEdLR0tVMPeCX?si=c68919fe62d9499d</t>
   </si>
   <si>
     <t>BuxWV 264</t>
@@ -2173,6 +2203,9 @@
 6. Allegro</t>
   </si>
   <si>
+    <t>https://open.spotify.com/track/23RsymnSa8BEbuUqnU8Ont?si=497b8360045f4eb0</t>
+  </si>
+  <si>
     <t>BuxWV 265</t>
   </si>
   <si>
@@ -2185,6 +2218,9 @@
 4. Vivace
 5. Largo
 6. Allegro</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/track/3TcjNdWfOZdWci8D8iw6Oz?si=4cb233c5a63847af</t>
   </si>
   <si>
     <t>BuxWV 266</t>
@@ -2980,7 +3016,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3526,10 +3562,10 @@
     <col min="4" max="4" width="13.5135135135135" style="2" customWidth="1"/>
     <col min="5" max="5" width="12.3513513513514" style="2" customWidth="1"/>
     <col min="6" max="6" width="18.5315315315315" style="2" customWidth="1"/>
-    <col min="7" max="7" width="32.972972972973" style="5" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="58.7657657657658" style="5" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="32.972972972973" style="5" customWidth="1"/>
+    <col min="8" max="8" width="58.7657657657658" style="5" customWidth="1"/>
     <col min="9" max="9" width="32.972972972973" style="5" customWidth="1"/>
-    <col min="10" max="10" width="20.9189189189189" style="5" customWidth="1"/>
+    <col min="10" max="10" width="20.9189189189189" style="4" customWidth="1"/>
     <col min="11" max="16384" width="8.61261261261261" style="5"/>
   </cols>
   <sheetData>
@@ -3561,7 +3597,7 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -8387,11 +8423,9 @@
       <c r="H262" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="I262" s="5" t="s">
+      <c r="I262" s="5"/>
+      <c r="J262" s="12" t="s">
         <v>634</v>
-      </c>
-      <c r="J262" s="12" t="s">
-        <v>635</v>
       </c>
     </row>
     <row r="263" customHeight="1" spans="1:10">
@@ -8399,10 +8433,10 @@
         <v>253</v>
       </c>
       <c r="B263" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="D263" s="2" t="s">
         <v>636</v>
-      </c>
-      <c r="D263" s="2" t="s">
-        <v>637</v>
       </c>
       <c r="E263" s="2" t="s">
         <v>631</v>
@@ -8411,10 +8445,13 @@
         <v>55</v>
       </c>
       <c r="G263" s="5" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H263" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J263" s="12" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="264" customHeight="1" spans="1:10">
@@ -8439,16 +8476,19 @@
       <c r="H264" s="5" t="s">
         <v>633</v>
       </c>
+      <c r="J264" s="12" t="s">
+        <v>642</v>
+      </c>
     </row>
     <row r="265" customHeight="1" spans="1:10">
       <c r="A265" s="7">
         <v>255</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E265" s="2" t="s">
         <v>631</v>
@@ -8457,10 +8497,13 @@
         <v>446</v>
       </c>
       <c r="G265" s="5" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="H265" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J265" s="12" t="s">
+        <v>646</v>
       </c>
     </row>
     <row r="266" customHeight="1" spans="1:10">
@@ -8468,10 +8511,10 @@
         <v>256</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="D266" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="E266" s="2" t="s">
         <v>631</v>
@@ -8480,10 +8523,13 @@
         <v>415</v>
       </c>
       <c r="G266" s="5" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="H266" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J266" s="12" t="s">
+        <v>650</v>
       </c>
     </row>
     <row r="267" customHeight="1" spans="1:10">
@@ -8491,10 +8537,10 @@
         <v>257</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="E267" s="2" t="s">
         <v>631</v>
@@ -8503,10 +8549,13 @@
         <v>423</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="H267" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J267" s="12" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="268" customHeight="1" spans="1:10">
@@ -8514,10 +8563,10 @@
         <v>258</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="D268" s="2" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="E268" s="2" t="s">
         <v>631</v>
@@ -8526,10 +8575,13 @@
         <v>427</v>
       </c>
       <c r="G268" s="5" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="H268" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J268" s="12" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="269" customHeight="1" spans="1:10">
@@ -8537,13 +8589,13 @@
         <v>259</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="C269" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D269" s="2" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="E269" s="2" t="s">
         <v>631</v>
@@ -8552,10 +8604,13 @@
         <v>446</v>
       </c>
       <c r="G269" s="5" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="H269" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J269" s="12" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="270" customHeight="1" spans="1:10">
@@ -8563,13 +8618,13 @@
         <v>260</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="C270" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D270" s="2" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="E270" s="2" t="s">
         <v>631</v>
@@ -8578,10 +8633,13 @@
         <v>421</v>
       </c>
       <c r="G270" s="5" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="H270" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J270" s="12" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="271" customHeight="1" spans="1:10">
@@ -8589,13 +8647,13 @@
         <v>261</v>
       </c>
       <c r="B271" s="3" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="C271" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D271" s="2" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="E271" s="2" t="s">
         <v>631</v>
@@ -8604,10 +8662,13 @@
         <v>436</v>
       </c>
       <c r="G271" s="5" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="H271" s="5" t="s">
         <v>633</v>
+      </c>
+      <c r="J271" s="12" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="272" customHeight="1" spans="1:10">
@@ -8615,13 +8676,13 @@
         <v>262</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="C272" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D272" s="2" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="E272" s="2" t="s">
         <v>631</v>
@@ -8630,24 +8691,27 @@
         <v>455</v>
       </c>
       <c r="G272" s="5" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="H272" s="5" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="273" customHeight="1" spans="1:9">
+      <c r="J272" s="12" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="273" customHeight="1" spans="1:10">
       <c r="A273" s="7">
         <v>263</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>667</v>
+        <v>676</v>
       </c>
       <c r="C273" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D273" s="2" t="s">
-        <v>668</v>
+        <v>677</v>
       </c>
       <c r="E273" s="2" t="s">
         <v>631</v>
@@ -8656,24 +8720,27 @@
         <v>440</v>
       </c>
       <c r="G273" s="5" t="s">
-        <v>669</v>
+        <v>678</v>
       </c>
       <c r="H273" s="5" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="274" customHeight="1" spans="1:9">
+      <c r="J273" s="12" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="274" customHeight="1" spans="1:10">
       <c r="A274" s="7">
         <v>264</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="C274" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D274" s="2" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
       <c r="E274" s="2" t="s">
         <v>631</v>
@@ -8682,24 +8749,27 @@
         <v>425</v>
       </c>
       <c r="G274" s="5" t="s">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="H274" s="5" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="275" customHeight="1" spans="1:9">
+      <c r="J274" s="12" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="275" customHeight="1" spans="1:10">
       <c r="A275" s="7">
         <v>265</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="C275" s="4" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="D275" s="2" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="E275" s="2" t="s">
         <v>631</v>
@@ -8708,18 +8778,21 @@
         <v>430</v>
       </c>
       <c r="G275" s="5" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="H275" s="5" t="s">
         <v>633</v>
       </c>
-    </row>
-    <row r="276" customHeight="1" spans="1:9">
+      <c r="J275" s="12" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="276" customHeight="1" spans="1:10">
       <c r="A276" s="7">
         <v>266</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>676</v>
+        <v>688</v>
       </c>
       <c r="E276" s="2" t="s">
         <v>631</v>
@@ -8728,18 +8801,18 @@
         <v>415</v>
       </c>
       <c r="G276" s="5" t="s">
-        <v>677</v>
+        <v>689</v>
       </c>
       <c r="H276" s="5" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="277" customHeight="1" spans="1:9">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="277" customHeight="1" spans="1:10">
       <c r="A277" s="7">
         <v>267</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>679</v>
+        <v>691</v>
       </c>
       <c r="E277" s="2" t="s">
         <v>631</v>
@@ -8748,18 +8821,18 @@
         <v>421</v>
       </c>
       <c r="G277" s="5" t="s">
-        <v>680</v>
+        <v>692</v>
       </c>
       <c r="H277" s="5" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="278" customHeight="1" spans="1:9">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="278" customHeight="1" spans="1:10">
       <c r="A278" s="7">
         <v>268</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>682</v>
+        <v>694</v>
       </c>
       <c r="E278" s="2" t="s">
         <v>631</v>
@@ -8768,18 +8841,18 @@
         <v>421</v>
       </c>
       <c r="G278" s="5" t="s">
-        <v>683</v>
+        <v>695</v>
       </c>
       <c r="H278" s="5" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="279" customHeight="1" spans="1:9">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="279" customHeight="1" spans="1:10">
       <c r="A279" s="7">
         <v>269</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>685</v>
+        <v>697</v>
       </c>
       <c r="E279" s="2" t="s">
         <v>631</v>
@@ -8788,18 +8861,18 @@
         <v>430</v>
       </c>
       <c r="G279" s="5" t="s">
-        <v>686</v>
+        <v>698</v>
       </c>
       <c r="H279" s="5" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="280" customHeight="1" spans="1:9">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="280" customHeight="1" spans="1:10">
       <c r="A280" s="7">
         <v>270</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>687</v>
+        <v>699</v>
       </c>
       <c r="E280" s="2" t="s">
         <v>631</v>
@@ -8808,18 +8881,18 @@
         <v>430</v>
       </c>
       <c r="H280" s="5" t="s">
-        <v>688</v>
+        <v>700</v>
       </c>
       <c r="I280" s="5" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="281" customHeight="1" spans="1:9">
+    <row r="281" customHeight="1" spans="1:10">
       <c r="A281" s="7">
         <v>271</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>689</v>
+        <v>701</v>
       </c>
       <c r="E281" s="2" t="s">
         <v>631</v>
@@ -8828,18 +8901,18 @@
         <v>55</v>
       </c>
       <c r="G281" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="H281" s="5" t="s">
         <v>690</v>
       </c>
-      <c r="H281" s="5" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="282" customHeight="1" spans="1:9">
+    </row>
+    <row r="282" customHeight="1" spans="1:10">
       <c r="A282" s="7">
         <v>272</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="E282" s="2" t="s">
         <v>631</v>
@@ -8848,18 +8921,18 @@
         <v>444</v>
       </c>
       <c r="G282" s="5" t="s">
-        <v>692</v>
+        <v>704</v>
       </c>
       <c r="H282" s="5" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="283" customHeight="1" spans="1:9">
+    <row r="283" customHeight="1" spans="1:10">
       <c r="A283" s="7">
         <v>273</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>693</v>
+        <v>705</v>
       </c>
       <c r="E283" s="2" t="s">
         <v>631</v>
@@ -8868,47 +8941,47 @@
         <v>446</v>
       </c>
       <c r="G283" s="5" t="s">
-        <v>694</v>
+        <v>706</v>
       </c>
       <c r="H283" s="5" t="s">
         <v>633</v>
       </c>
       <c r="I283" s="5" t="s">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="284" customHeight="1" spans="1:9">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="284" customHeight="1" spans="1:10">
       <c r="A284" s="7">
         <v>274</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>696</v>
+        <v>708</v>
       </c>
       <c r="C284" s="4" t="s">
-        <v>697</v>
+        <v>709</v>
       </c>
       <c r="E284" s="2" t="s">
         <v>631</v>
       </c>
       <c r="I284" s="5" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="285" customHeight="1" spans="1:9">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="285" customHeight="1" spans="1:10">
       <c r="A285" s="7">
         <v>275</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="C285" s="4" t="s">
-        <v>700</v>
+        <v>712</v>
       </c>
       <c r="E285" s="2" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="I285" s="5" t="s">
-        <v>698</v>
+        <v>710</v>
       </c>
     </row>
   </sheetData>
@@ -8923,6 +8996,19 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="J262" r:id="rId1" display="https://open.spotify.com/track/5V2jyo36dQEe0p4Cz9E8ci?si=847f7f58ae0045d0"/>
+    <hyperlink ref="J263" r:id="rId2" display="https://open.spotify.com/track/2aQJ1oNCXSL9XWiTuUnUh5?si=fd373831f91c4d53"/>
+    <hyperlink ref="J264" r:id="rId3" display="https://open.spotify.com/track/0FbNGIBKxiHuNKHwBVa3KV?si=be7fa4ab5bb44070"/>
+    <hyperlink ref="J265" r:id="rId4" display="https://open.spotify.com/track/41snipsr88aJQUoHA5QzG3?si=85e3ec6881d14bfe"/>
+    <hyperlink ref="J266" r:id="rId5" display="https://open.spotify.com/track/66Oq6njsbUCZu399cheY4q?si=3c2a19e57f834507"/>
+    <hyperlink ref="J267" r:id="rId6" display="https://open.spotify.com/track/2A4yXz2VhLVEBHAv4EdEBv?si=351ec16a12b242af"/>
+    <hyperlink ref="J268" r:id="rId7" display="https://open.spotify.com/track/0duf649xp9xw84aBwPsHKY?si=072c6e1d5f534488"/>
+    <hyperlink ref="J269" r:id="rId8" display="https://open.spotify.com/track/2MeB6etCEHNZixEffMDHV1?si=225bb02889a14429"/>
+    <hyperlink ref="J270" r:id="rId9" display="https://open.spotify.com/track/1huvSof1V0V73f5FpE5RSI?si=9e8cb98ea5bc443c"/>
+    <hyperlink ref="J271" r:id="rId10" display="https://open.spotify.com/track/3I9g7jkYe5sdW7DpIPdm55?si=d470f7acbb2640f2"/>
+    <hyperlink ref="J272" r:id="rId11" display="https://open.spotify.com/track/3cBHUIZF9bPmf4DxkjOheq?si=f72f8f4b9f09441b"/>
+    <hyperlink ref="J273" r:id="rId12" display="https://open.spotify.com/track/2C5lNDTCyHEdLR0tVMPeCX?si=c68919fe62d9499d"/>
+    <hyperlink ref="J274" r:id="rId13" display="https://open.spotify.com/track/23RsymnSa8BEbuUqnU8Ont?si=497b8360045f4eb0"/>
+    <hyperlink ref="J275" r:id="rId14" display="https://open.spotify.com/track/3TcjNdWfOZdWci8D8iw6Oz?si=4cb233c5a63847af"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
data: update BuxWV, CPE, Corelli
</commit_message>
<xml_diff>
--- a/xlsx/BuxWV.xlsx
+++ b/xlsx/BuxWV.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="766">
   <si>
     <t>SORT</t>
   </si>
@@ -2049,6 +2049,9 @@
   </si>
   <si>
     <t>Courant zimble (8 variations)</t>
+  </si>
+  <si>
+    <t>Keyboard Variation</t>
   </si>
   <si>
     <t>BuxWV 246</t>
@@ -8613,6 +8616,9 @@
       <c r="C255" s="4" t="s">
         <v>652</v>
       </c>
+      <c r="E255" s="2" t="s">
+        <v>653</v>
+      </c>
       <c r="F255" s="2" t="s">
         <v>455</v>
       </c>
@@ -8625,10 +8631,13 @@
         <v>246</v>
       </c>
       <c r="B256" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="C256" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="E256" s="2" t="s">
         <v>653</v>
-      </c>
-      <c r="C256" s="4" t="s">
-        <v>654</v>
       </c>
       <c r="F256" s="2" t="s">
         <v>416</v>
@@ -8642,10 +8651,13 @@
         <v>247</v>
       </c>
       <c r="B257" s="3" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C257" s="4" t="s">
-        <v>656</v>
+        <v>657</v>
+      </c>
+      <c r="E257" s="2" t="s">
+        <v>653</v>
       </c>
       <c r="F257" s="2" t="s">
         <v>416</v>
@@ -8659,10 +8671,13 @@
         <v>248</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C258" s="4" t="s">
-        <v>658</v>
+        <v>659</v>
+      </c>
+      <c r="E258" s="2" t="s">
+        <v>653</v>
       </c>
       <c r="F258" s="2" t="s">
         <v>455</v>
@@ -8676,10 +8691,13 @@
         <v>249</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C259" s="4" t="s">
-        <v>660</v>
+        <v>661</v>
+      </c>
+      <c r="E259" s="2" t="s">
+        <v>653</v>
       </c>
       <c r="F259" s="2" t="s">
         <v>455</v>
@@ -8693,10 +8711,13 @@
         <v>250</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C260" s="5" t="s">
-        <v>662</v>
+        <v>663</v>
+      </c>
+      <c r="E260" s="2" t="s">
+        <v>653</v>
       </c>
       <c r="F260" s="2" t="s">
         <v>55</v>
@@ -8710,10 +8731,10 @@
         <v>251</v>
       </c>
       <c r="B261" s="3" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C261" s="4" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E261" s="2" t="s">
         <v>607</v>
@@ -8722,7 +8743,7 @@
         <v>609</v>
       </c>
       <c r="I261" s="5" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
     </row>
     <row r="262" customHeight="1" spans="1:10">
@@ -8730,28 +8751,28 @@
         <v>252</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C262" s="4" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E262" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F262" s="2" t="s">
         <v>436</v>
       </c>
       <c r="G262" s="5" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="H262" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J262" s="12" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="263" customHeight="1" spans="1:10">
@@ -8759,28 +8780,28 @@
         <v>253</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C263" s="4" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="D263" s="2" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="E263" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F263" s="2" t="s">
         <v>55</v>
       </c>
       <c r="G263" s="5" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="H263" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J263" s="12" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
     </row>
     <row r="264" customHeight="1" spans="1:10">
@@ -8788,28 +8809,28 @@
         <v>254</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C264" s="4" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="E264" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F264" s="2" t="s">
         <v>455</v>
       </c>
       <c r="G264" s="5" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="H264" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J264" s="12" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="265" customHeight="1" spans="1:10">
@@ -8817,28 +8838,28 @@
         <v>255</v>
       </c>
       <c r="B265" s="3" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C265" s="4" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E265" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F265" s="2" t="s">
         <v>458</v>
       </c>
       <c r="G265" s="5" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="H265" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J265" s="12" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="266" customHeight="1" spans="1:10">
@@ -8846,28 +8867,28 @@
         <v>256</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C266" s="4" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D266" s="2" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="E266" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F266" s="2" t="s">
         <v>416</v>
       </c>
       <c r="G266" s="5" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="H266" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J266" s="12" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
     </row>
     <row r="267" customHeight="1" spans="1:10">
@@ -8875,28 +8896,28 @@
         <v>257</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C267" s="4" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="E267" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F267" s="2" t="s">
         <v>426</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="H267" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J267" s="12" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
     </row>
     <row r="268" customHeight="1" spans="1:10">
@@ -8904,28 +8925,28 @@
         <v>258</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C268" s="4" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D268" s="2" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E268" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F268" s="2" t="s">
         <v>432</v>
       </c>
       <c r="G268" s="5" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H268" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J268" s="12" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
     </row>
     <row r="269" customHeight="1" spans="1:10">
@@ -8933,28 +8954,28 @@
         <v>259</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C269" s="4" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D269" s="2" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="E269" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F269" s="2" t="s">
         <v>458</v>
       </c>
       <c r="G269" s="5" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H269" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J269" s="12" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
     </row>
     <row r="270" customHeight="1" spans="1:10">
@@ -8962,28 +8983,28 @@
         <v>260</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C270" s="4" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D270" s="2" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="E270" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F270" s="2" t="s">
         <v>423</v>
       </c>
       <c r="G270" s="5" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="H270" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J270" s="12" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
     </row>
     <row r="271" customHeight="1" spans="1:10">
@@ -8991,28 +9012,28 @@
         <v>261</v>
       </c>
       <c r="B271" s="3" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C271" s="4" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D271" s="2" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="E271" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F271" s="2" t="s">
         <v>445</v>
       </c>
       <c r="G271" s="5" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="H271" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J271" s="12" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
     </row>
     <row r="272" customHeight="1" spans="1:10">
@@ -9020,28 +9041,28 @@
         <v>262</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C272" s="4" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="D272" s="2" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="E272" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F272" s="2" t="s">
         <v>470</v>
       </c>
       <c r="G272" s="5" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="H272" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J272" s="12" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="273" customHeight="1" spans="1:10">
@@ -9049,28 +9070,28 @@
         <v>263</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C273" s="4" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D273" s="2" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E273" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F273" s="2" t="s">
         <v>450</v>
       </c>
       <c r="G273" s="5" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="H273" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J273" s="12" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
     </row>
     <row r="274" customHeight="1" spans="1:10">
@@ -9078,28 +9099,28 @@
         <v>264</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C274" s="4" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="D274" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E274" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F274" s="2" t="s">
         <v>429</v>
       </c>
       <c r="G274" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="H274" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J274" s="12" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
     </row>
     <row r="275" customHeight="1" spans="1:10">
@@ -9107,28 +9128,28 @@
         <v>265</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C275" s="4" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="D275" s="2" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E275" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F275" s="2" t="s">
         <v>436</v>
       </c>
       <c r="G275" s="5" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H275" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="J275" s="12" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
     </row>
     <row r="276" customHeight="1" spans="1:10">
@@ -9136,22 +9157,22 @@
         <v>266</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C276" s="4" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E276" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F276" s="2" t="s">
         <v>416</v>
       </c>
       <c r="G276" s="5" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="H276" s="5" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="277" customHeight="1" spans="1:10">
@@ -9159,22 +9180,22 @@
         <v>267</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C277" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="E277" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F277" s="2" t="s">
         <v>423</v>
       </c>
       <c r="G277" s="5" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="H277" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="278" customHeight="1" spans="1:10">
@@ -9182,22 +9203,22 @@
         <v>268</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C278" s="4" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="E278" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F278" s="2" t="s">
         <v>423</v>
       </c>
       <c r="G278" s="5" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="H278" s="5" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
     </row>
     <row r="279" customHeight="1" spans="1:10">
@@ -9205,22 +9226,22 @@
         <v>269</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C279" s="4" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="E279" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F279" s="2" t="s">
         <v>436</v>
       </c>
       <c r="G279" s="5" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="H279" s="5" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="280" customHeight="1" spans="1:10">
@@ -9228,19 +9249,19 @@
         <v>270</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C280" s="4" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="E280" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F280" s="2" t="s">
         <v>436</v>
       </c>
       <c r="H280" s="5" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="I280" s="5" t="s">
         <v>285</v>
@@ -9251,22 +9272,22 @@
         <v>271</v>
       </c>
       <c r="B281" s="3" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="C281" s="4" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="E281" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F281" s="2" t="s">
         <v>55</v>
       </c>
       <c r="G281" s="5" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="H281" s="5" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="282" customHeight="1" spans="1:10">
@@ -9274,22 +9295,22 @@
         <v>272</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C282" s="4" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E282" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F282" s="2" t="s">
         <v>455</v>
       </c>
       <c r="G282" s="5" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="H282" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
     </row>
     <row r="283" customHeight="1" spans="1:10">
@@ -9297,25 +9318,25 @@
         <v>273</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C283" s="4" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E283" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F283" s="2" t="s">
         <v>458</v>
       </c>
       <c r="G283" s="5" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="H283" s="5" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="I283" s="5" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
     </row>
     <row r="284" customHeight="1" spans="1:10">
@@ -9323,17 +9344,16 @@
         <v>274</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>759</v>
-      </c>
-      <c r="C284" s="4"/>
+        <v>760</v>
+      </c>
       <c r="E284" s="2" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="H284" s="5" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="I284" s="5" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
     </row>
     <row r="285" customHeight="1" spans="1:10">
@@ -9341,16 +9361,16 @@
         <v>275</v>
       </c>
       <c r="B285" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="C285" s="4" t="s">
+        <v>764</v>
+      </c>
+      <c r="E285" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="I285" s="5" t="s">
         <v>762</v>
-      </c>
-      <c r="C285" s="4" t="s">
-        <v>763</v>
-      </c>
-      <c r="E285" s="2" t="s">
-        <v>764</v>
-      </c>
-      <c r="I285" s="5" t="s">
-        <v>761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>